<commit_message>
tests: updated test data
</commit_message>
<xml_diff>
--- a/tests/data/_schema/physical/car_dms_rules.xlsx
+++ b/tests/data/_schema/physical/car_dms_rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikola/Repos/neat/tests/data/_schema/physical/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AndersAlbert\Projects\main\neat\tests\data\_schema\physical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87C31E1-F3AA-7549-8BB1-7B9DC6D96D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713AA20B-B3DB-4AE7-84B9-BC30EEC1738C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="42700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -126,9 +126,6 @@
     <t>make</t>
   </si>
   <si>
-    <t>edge(type=Car.Manufacturer)</t>
-  </si>
-  <si>
     <t>Manufacturer</t>
   </si>
   <si>
@@ -244,6 +241,9 @@
   </si>
   <si>
     <t>conceptual</t>
+  </si>
+  <si>
+    <t>edge(type=make)</t>
   </si>
 </sst>
 </file>
@@ -253,7 +253,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -624,13 +624,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="26.5" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="15.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -638,7 +638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="15.75">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -646,7 +646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="15.75">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -654,7 +654,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="15.75">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -662,17 +662,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ht="15.75">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" ht="15.75">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" ht="15.75">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -680,7 +680,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" ht="15.75">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -688,7 +688,7 @@
         <v>45695.809878616063</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" ht="15.75">
       <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
@@ -696,14 +696,14 @@
         <v>45695.809878616303</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" ht="15.75">
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" ht="15.75">
       <c r="A11" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -714,21 +714,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="34.5" customWidth="1"/>
-    <col min="2" max="2" width="13.5" customWidth="1"/>
+    <col min="1" max="1" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" customWidth="1"/>
     <col min="3" max="4" width="13" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="27.5" customWidth="1"/>
+    <col min="5" max="5" width="27.42578125" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
     <col min="7" max="11" width="13" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="18.5" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="18.42578125" hidden="1" customWidth="1"/>
     <col min="13" max="14" width="13" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="94.6640625" customWidth="1"/>
+    <col min="15" max="15" width="94.7109375" customWidth="1"/>
     <col min="16" max="16" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="26.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -747,7 +747,7 @@
       <c r="N1" s="4"/>
       <c r="O1" s="4"/>
     </row>
-    <row r="2" spans="1:16" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="18.75">
       <c r="A2" s="5" t="s">
         <v>16</v>
       </c>
@@ -791,13 +791,13 @@
         <v>29</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P2" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="15.75">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -805,30 +805,30 @@
         <v>32</v>
       </c>
       <c r="E3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" t="s">
         <v>33</v>
-      </c>
-      <c r="F3" t="s">
-        <v>34</v>
       </c>
       <c r="I3" t="b">
         <v>1</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="15.75">
       <c r="A4" t="s">
         <v>31</v>
       </c>
       <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s">
         <v>36</v>
-      </c>
-      <c r="F4" t="s">
-        <v>37</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -843,27 +843,27 @@
         <v>31</v>
       </c>
       <c r="L4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="P4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="15.75">
       <c r="A5" t="s">
         <v>31</v>
       </c>
       <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s">
         <v>39</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>40</v>
-      </c>
-      <c r="F5" t="s">
-        <v>41</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -878,24 +878,24 @@
         <v>31</v>
       </c>
       <c r="L5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="15.75">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -907,27 +907,27 @@
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L6" t="s">
         <v>8</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="15.75">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
@@ -939,16 +939,16 @@
         <v>0</v>
       </c>
       <c r="K7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L7" t="s">
         <v>8</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="P7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -960,17 +960,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.5" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
     <col min="2" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="79.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="79.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="26.25">
       <c r="A1" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -980,7 +980,7 @@
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
     </row>
-    <row r="2" spans="1:8" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="18.75">
       <c r="A2" s="5" t="s">
         <v>16</v>
       </c>
@@ -991,22 +991,22 @@
         <v>19</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>49</v>
-      </c>
       <c r="G2" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="15.75">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -1014,38 +1014,38 @@
         <v>1</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1057,15 +1057,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.5" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
     <col min="2" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="26.25">
       <c r="A1" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -1073,7 +1073,7 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
     </row>
-    <row r="2" spans="1:6" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="18.75">
       <c r="A2" s="5" t="s">
         <v>26</v>
       </c>
@@ -1087,25 +1087,25 @@
         <v>29</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1116,28 +1116,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.5" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" customWidth="1"/>
     <col min="2" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="13" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="26.25">
       <c r="A1" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
     </row>
-    <row r="2" spans="1:5" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="18.75">
       <c r="A2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>57</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>18</v>
@@ -1157,28 +1157,28 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.5" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
     <col min="2" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="13" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="26.25">
       <c r="A1" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
     </row>
-    <row r="2" spans="1:5" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="18.75">
       <c r="A2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>18</v>
@@ -1190,12 +1190,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" t="s">
         <v>61</v>
-      </c>
-      <c r="B3" t="s">
-        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>